<commit_message>
How To Run PHP , PHP with Database
</commit_message>
<xml_diff>
--- a/MINI PROJECT/3IST02_Mini Project Details.xlsx
+++ b/MINI PROJECT/3IST02_Mini Project Details.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="291">
   <si>
     <t>SI.NO</t>
   </si>
@@ -939,6 +939,15 @@
   </si>
   <si>
     <t>20241IST0126(lead)</t>
+  </si>
+  <si>
+    <t>PPT</t>
+  </si>
+  <si>
+    <t>SUBMITTED</t>
+  </si>
+  <si>
+    <t>NOT SUBMITTED</t>
   </si>
 </sst>
 </file>
@@ -1128,7 +1137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1169,7 +1178,7 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1179,16 +1188,31 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1470,16 +1494,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P67"/>
+  <dimension ref="A1:Q67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="7" max="7" width="35.28515625" customWidth="1"/>
-    <col min="8" max="8" width="69.42578125" customWidth="1"/>
-    <col min="9" max="9" width="43.7109375" customWidth="1"/>
+    <col min="7" max="8" width="19.42578125" customWidth="1"/>
+    <col min="9" max="9" width="44.140625" customWidth="1"/>
+    <col min="10" max="10" width="43.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75">
+    <row r="1" spans="1:10" ht="15.75">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1499,13 +1523,16 @@
         <v>263</v>
       </c>
       <c r="H1" s="20" t="s">
+        <v>288</v>
+      </c>
+      <c r="I1" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="J1" s="20" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="30" customHeight="1">
+    <row r="2" spans="1:10" ht="30" customHeight="1">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1522,17 +1549,20 @@
         <v>6</v>
       </c>
       <c r="F2" s="17"/>
-      <c r="G2" s="27" t="s">
+      <c r="G2" s="24" t="s">
         <v>242</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="I2" s="25" t="s">
         <v>267</v>
       </c>
-      <c r="I2" s="24" t="s">
+      <c r="J2" s="29" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75">
+    <row r="3" spans="1:10" ht="15.75">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1549,11 +1579,12 @@
         <v>10</v>
       </c>
       <c r="F3" s="17"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="24"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.75">
+      <c r="G3" s="24"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="29"/>
+    </row>
+    <row r="4" spans="1:10" ht="15.75">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1570,11 +1601,12 @@
         <v>14</v>
       </c>
       <c r="F4" s="17"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="24"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.75">
+      <c r="G4" s="24"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="29"/>
+    </row>
+    <row r="5" spans="1:10" ht="15.75">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1591,11 +1623,12 @@
         <v>18</v>
       </c>
       <c r="F5" s="17"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="24"/>
-    </row>
-    <row r="6" spans="1:9" ht="70.5" customHeight="1">
+      <c r="G5" s="24"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="29"/>
+    </row>
+    <row r="6" spans="1:10" ht="70.5" customHeight="1">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -1611,11 +1644,12 @@
       <c r="E6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="27"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="24"/>
-    </row>
-    <row r="7" spans="1:9" ht="15.75">
+      <c r="G6" s="24"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="29"/>
+    </row>
+    <row r="7" spans="1:10" ht="15.75">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1632,15 +1666,18 @@
         <v>26</v>
       </c>
       <c r="F7" s="17"/>
-      <c r="G7" s="30" t="s">
+      <c r="G7" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="H7" s="28" t="s">
+      <c r="H7" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="I7" s="27" t="s">
         <v>268</v>
       </c>
-      <c r="I7" s="24"/>
-    </row>
-    <row r="8" spans="1:9" ht="15.75">
+      <c r="J7" s="29"/>
+    </row>
+    <row r="8" spans="1:10" ht="15.75">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1657,11 +1694,12 @@
         <v>28</v>
       </c>
       <c r="F8" s="17"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="24"/>
-    </row>
-    <row r="9" spans="1:9" ht="15.75">
+      <c r="G8" s="24"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="29"/>
+    </row>
+    <row r="9" spans="1:10" ht="15.75">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1678,11 +1716,12 @@
         <v>31</v>
       </c>
       <c r="F9" s="17"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="24"/>
-    </row>
-    <row r="10" spans="1:9" ht="15.75">
+      <c r="G9" s="24"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="29"/>
+    </row>
+    <row r="10" spans="1:10" ht="15.75">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1699,11 +1738,12 @@
         <v>35</v>
       </c>
       <c r="F10" s="17"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="24"/>
-    </row>
-    <row r="11" spans="1:9" ht="72.75" customHeight="1">
+      <c r="G10" s="24"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="29"/>
+    </row>
+    <row r="11" spans="1:10" ht="72.75" customHeight="1">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1720,11 +1760,12 @@
         <v>39</v>
       </c>
       <c r="F11" s="17"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="24"/>
-    </row>
-    <row r="12" spans="1:9" ht="15.75">
+      <c r="G11" s="24"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="29"/>
+    </row>
+    <row r="12" spans="1:10" ht="15.75">
       <c r="A12" s="8">
         <v>11</v>
       </c>
@@ -1741,15 +1782,18 @@
         <v>43</v>
       </c>
       <c r="F12" s="17"/>
-      <c r="G12" s="30" t="s">
+      <c r="G12" s="24" t="s">
         <v>244</v>
       </c>
-      <c r="H12" s="25" t="s">
+      <c r="H12" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="I12" s="25" t="s">
         <v>269</v>
       </c>
-      <c r="I12" s="24"/>
-    </row>
-    <row r="13" spans="1:9" ht="15.75">
+      <c r="J12" s="29"/>
+    </row>
+    <row r="13" spans="1:10" ht="15.75">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1766,11 +1810,12 @@
         <v>47</v>
       </c>
       <c r="F13" s="17"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="24"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.75">
+      <c r="G13" s="24"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="29"/>
+    </row>
+    <row r="14" spans="1:10" ht="15.75">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1787,11 +1832,12 @@
         <v>51</v>
       </c>
       <c r="F14" s="17"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="24"/>
-    </row>
-    <row r="15" spans="1:9" ht="15.75">
+      <c r="G14" s="24"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="29"/>
+    </row>
+    <row r="15" spans="1:10" ht="15.75">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1808,11 +1854,12 @@
         <v>53</v>
       </c>
       <c r="F15" s="17"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="24"/>
-    </row>
-    <row r="16" spans="1:9" ht="89.25" customHeight="1">
+      <c r="G15" s="24"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="29"/>
+    </row>
+    <row r="16" spans="1:10" ht="89.25" customHeight="1">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1829,11 +1876,12 @@
         <v>57</v>
       </c>
       <c r="F16" s="17"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="24"/>
-    </row>
-    <row r="17" spans="1:9" ht="15.75">
+      <c r="G16" s="24"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="29"/>
+    </row>
+    <row r="17" spans="1:10" ht="15.75">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1850,15 +1898,18 @@
         <v>60</v>
       </c>
       <c r="F17" s="17"/>
-      <c r="G17" s="30" t="s">
+      <c r="G17" s="24" t="s">
         <v>245</v>
       </c>
-      <c r="H17" s="25" t="s">
+      <c r="H17" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="I17" s="25" t="s">
         <v>270</v>
       </c>
-      <c r="I17" s="24"/>
-    </row>
-    <row r="18" spans="1:9" ht="15.75">
+      <c r="J17" s="29"/>
+    </row>
+    <row r="18" spans="1:10" ht="15.75">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1875,11 +1926,12 @@
         <v>63</v>
       </c>
       <c r="F18" s="17"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="24"/>
-    </row>
-    <row r="19" spans="1:9" ht="15.75">
+      <c r="G18" s="24"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="29"/>
+    </row>
+    <row r="19" spans="1:10" ht="15.75">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1896,11 +1948,12 @@
         <v>67</v>
       </c>
       <c r="F19" s="17"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="24"/>
-    </row>
-    <row r="20" spans="1:9" ht="15.75">
+      <c r="G19" s="24"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="26"/>
+      <c r="J19" s="29"/>
+    </row>
+    <row r="20" spans="1:10" ht="15.75">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1917,11 +1970,12 @@
         <v>71</v>
       </c>
       <c r="F20" s="17"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="24"/>
-    </row>
-    <row r="21" spans="1:9" ht="61.5" customHeight="1">
+      <c r="G20" s="24"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="29"/>
+    </row>
+    <row r="21" spans="1:10" ht="61.5" customHeight="1">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1938,11 +1992,12 @@
         <v>75</v>
       </c>
       <c r="F21" s="17"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="24"/>
-    </row>
-    <row r="22" spans="1:9" ht="15.75">
+      <c r="G21" s="24"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="29"/>
+    </row>
+    <row r="22" spans="1:10" ht="15.75">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1959,15 +2014,18 @@
         <v>77</v>
       </c>
       <c r="F22" s="17"/>
-      <c r="G22" s="30" t="s">
+      <c r="G22" s="24" t="s">
         <v>246</v>
       </c>
-      <c r="H22" s="25" t="s">
+      <c r="H22" s="30" t="s">
+        <v>290</v>
+      </c>
+      <c r="I22" s="25" t="s">
         <v>271</v>
       </c>
-      <c r="I22" s="24"/>
-    </row>
-    <row r="23" spans="1:9" ht="15.75">
+      <c r="J22" s="29"/>
+    </row>
+    <row r="23" spans="1:10" ht="15.75">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1984,11 +2042,12 @@
         <v>81</v>
       </c>
       <c r="F23" s="17"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="24"/>
-    </row>
-    <row r="24" spans="1:9" ht="15.75">
+      <c r="G23" s="24"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="29"/>
+    </row>
+    <row r="24" spans="1:10" ht="15.75">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -2005,11 +2064,12 @@
         <v>85</v>
       </c>
       <c r="F24" s="17"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="26"/>
-      <c r="I24" s="24"/>
-    </row>
-    <row r="25" spans="1:9" ht="15.75">
+      <c r="G24" s="24"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="29"/>
+    </row>
+    <row r="25" spans="1:10" ht="15.75">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -2026,11 +2086,12 @@
         <v>89</v>
       </c>
       <c r="F25" s="17"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="24"/>
-    </row>
-    <row r="26" spans="1:9" ht="64.5" customHeight="1">
+      <c r="G25" s="24"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="29"/>
+    </row>
+    <row r="26" spans="1:10" ht="64.5" customHeight="1">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -2047,11 +2108,12 @@
         <v>93</v>
       </c>
       <c r="F26" s="17"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="24"/>
-    </row>
-    <row r="27" spans="1:9" ht="15.75">
+      <c r="G26" s="24"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="29"/>
+    </row>
+    <row r="27" spans="1:10" ht="15.75">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -2068,15 +2130,18 @@
         <v>97</v>
       </c>
       <c r="F27" s="17"/>
-      <c r="G27" s="30" t="s">
+      <c r="G27" s="24" t="s">
         <v>247</v>
       </c>
-      <c r="H27" s="25" t="s">
+      <c r="H27" s="30" t="s">
+        <v>290</v>
+      </c>
+      <c r="I27" s="25" t="s">
         <v>273</v>
       </c>
-      <c r="I27" s="24"/>
-    </row>
-    <row r="28" spans="1:9" ht="15.75">
+      <c r="J27" s="29"/>
+    </row>
+    <row r="28" spans="1:10" ht="15.75">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -2093,11 +2158,12 @@
         <v>101</v>
       </c>
       <c r="F28" s="17"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="24"/>
-    </row>
-    <row r="29" spans="1:9" ht="15.75">
+      <c r="G28" s="24"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="26"/>
+      <c r="J28" s="29"/>
+    </row>
+    <row r="29" spans="1:10" ht="15.75">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -2114,11 +2180,12 @@
         <v>105</v>
       </c>
       <c r="F29" s="17"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="24"/>
-    </row>
-    <row r="30" spans="1:9" ht="15.75">
+      <c r="G29" s="24"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="26"/>
+      <c r="J29" s="29"/>
+    </row>
+    <row r="30" spans="1:10" ht="15.75">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -2135,11 +2202,12 @@
         <v>107</v>
       </c>
       <c r="F30" s="17"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="24"/>
-    </row>
-    <row r="31" spans="1:9" ht="15.75">
+      <c r="G30" s="24"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="29"/>
+    </row>
+    <row r="31" spans="1:10" ht="15.75">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -2156,11 +2224,12 @@
         <v>111</v>
       </c>
       <c r="F31" s="17"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="24"/>
-    </row>
-    <row r="32" spans="1:9" ht="35.25" customHeight="1">
+      <c r="G31" s="24"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="26"/>
+      <c r="J31" s="29"/>
+    </row>
+    <row r="32" spans="1:10" ht="35.25" customHeight="1">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -2177,11 +2246,12 @@
         <v>115</v>
       </c>
       <c r="F32" s="17"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="24"/>
-    </row>
-    <row r="33" spans="1:16" ht="15.75">
+      <c r="G32" s="24"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="26"/>
+      <c r="J32" s="29"/>
+    </row>
+    <row r="33" spans="1:17" ht="15.75">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -2198,15 +2268,18 @@
         <v>119</v>
       </c>
       <c r="F33" s="17"/>
-      <c r="G33" s="30" t="s">
+      <c r="G33" s="24" t="s">
         <v>248</v>
       </c>
-      <c r="H33" s="25" t="s">
+      <c r="H33" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="I33" s="25" t="s">
         <v>274</v>
       </c>
-      <c r="I33" s="24"/>
-    </row>
-    <row r="34" spans="1:16" ht="15.75">
+      <c r="J33" s="29"/>
+    </row>
+    <row r="34" spans="1:17" ht="15.75">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -2223,11 +2296,12 @@
         <v>123</v>
       </c>
       <c r="F34" s="17"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="24"/>
-    </row>
-    <row r="35" spans="1:16" ht="15.75">
+      <c r="G34" s="24"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="26"/>
+      <c r="J34" s="29"/>
+    </row>
+    <row r="35" spans="1:17" ht="15.75">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -2244,11 +2318,12 @@
         <v>127</v>
       </c>
       <c r="F35" s="17"/>
-      <c r="G35" s="30"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="24"/>
-    </row>
-    <row r="36" spans="1:16" ht="15.75">
+      <c r="G35" s="24"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="26"/>
+      <c r="J35" s="29"/>
+    </row>
+    <row r="36" spans="1:17" ht="15.75">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -2265,18 +2340,19 @@
         <v>131</v>
       </c>
       <c r="F36" s="18"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="24"/>
-      <c r="J36" s="6"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="26"/>
+      <c r="J36" s="29"/>
       <c r="K36" s="6"/>
       <c r="L36" s="6"/>
       <c r="M36" s="6"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6"/>
       <c r="P36" s="6"/>
-    </row>
-    <row r="37" spans="1:16" ht="77.25" customHeight="1">
+      <c r="Q36" s="6"/>
+    </row>
+    <row r="37" spans="1:17" ht="77.25" customHeight="1">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -2293,11 +2369,12 @@
         <v>135</v>
       </c>
       <c r="F37" s="17"/>
-      <c r="G37" s="30"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="24"/>
-    </row>
-    <row r="38" spans="1:16" ht="15.75">
+      <c r="G37" s="24"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="26"/>
+      <c r="J37" s="29"/>
+    </row>
+    <row r="38" spans="1:17" ht="15.75">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -2314,15 +2391,18 @@
         <v>138</v>
       </c>
       <c r="F38" s="17"/>
-      <c r="G38" s="30" t="s">
+      <c r="G38" s="24" t="s">
         <v>249</v>
       </c>
-      <c r="H38" s="25" t="s">
+      <c r="H38" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="I38" s="25" t="s">
         <v>275</v>
       </c>
-      <c r="I38" s="24"/>
-    </row>
-    <row r="39" spans="1:16" ht="15.75">
+      <c r="J38" s="29"/>
+    </row>
+    <row r="39" spans="1:17" ht="15.75">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -2339,11 +2419,12 @@
         <v>142</v>
       </c>
       <c r="F39" s="17"/>
-      <c r="G39" s="30"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="24"/>
-    </row>
-    <row r="40" spans="1:16" ht="15.75">
+      <c r="G39" s="24"/>
+      <c r="H39" s="31"/>
+      <c r="I39" s="26"/>
+      <c r="J39" s="29"/>
+    </row>
+    <row r="40" spans="1:17" ht="15.75">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -2360,11 +2441,12 @@
         <v>146</v>
       </c>
       <c r="F40" s="17"/>
-      <c r="G40" s="30"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="24"/>
-    </row>
-    <row r="41" spans="1:16" ht="15.75">
+      <c r="G40" s="24"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="26"/>
+      <c r="J40" s="29"/>
+    </row>
+    <row r="41" spans="1:17" ht="15.75">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -2381,11 +2463,12 @@
         <v>150</v>
       </c>
       <c r="F41" s="17"/>
-      <c r="G41" s="30"/>
-      <c r="H41" s="26"/>
-      <c r="I41" s="24"/>
-    </row>
-    <row r="42" spans="1:16" ht="61.5" customHeight="1">
+      <c r="G41" s="24"/>
+      <c r="H41" s="31"/>
+      <c r="I41" s="26"/>
+      <c r="J41" s="29"/>
+    </row>
+    <row r="42" spans="1:17" ht="61.5" customHeight="1">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -2402,11 +2485,12 @@
         <v>154</v>
       </c>
       <c r="F42" s="17"/>
-      <c r="G42" s="30"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="24"/>
-    </row>
-    <row r="43" spans="1:16" ht="15.75">
+      <c r="G42" s="24"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="26"/>
+      <c r="J42" s="29"/>
+    </row>
+    <row r="43" spans="1:17" ht="15.75">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -2423,15 +2507,18 @@
         <v>158</v>
       </c>
       <c r="F43" s="17"/>
-      <c r="G43" s="30" t="s">
+      <c r="G43" s="24" t="s">
         <v>250</v>
       </c>
-      <c r="H43" s="25" t="s">
+      <c r="H43" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="I43" s="25" t="s">
         <v>276</v>
       </c>
-      <c r="I43" s="24"/>
-    </row>
-    <row r="44" spans="1:16" ht="15.75">
+      <c r="J43" s="29"/>
+    </row>
+    <row r="44" spans="1:17" ht="15.75">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -2448,11 +2535,12 @@
         <v>162</v>
       </c>
       <c r="F44" s="17"/>
-      <c r="G44" s="30"/>
-      <c r="H44" s="26"/>
-      <c r="I44" s="24"/>
-    </row>
-    <row r="45" spans="1:16" ht="15.75">
+      <c r="G44" s="24"/>
+      <c r="H44" s="31"/>
+      <c r="I44" s="26"/>
+      <c r="J44" s="29"/>
+    </row>
+    <row r="45" spans="1:17" ht="15.75">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -2469,11 +2557,12 @@
         <v>166</v>
       </c>
       <c r="F45" s="17"/>
-      <c r="G45" s="30"/>
-      <c r="H45" s="26"/>
-      <c r="I45" s="24"/>
-    </row>
-    <row r="46" spans="1:16" ht="15.75">
+      <c r="G45" s="24"/>
+      <c r="H45" s="31"/>
+      <c r="I45" s="26"/>
+      <c r="J45" s="29"/>
+    </row>
+    <row r="46" spans="1:17" ht="15.75">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -2490,11 +2579,12 @@
         <v>170</v>
       </c>
       <c r="F46" s="17"/>
-      <c r="G46" s="30"/>
-      <c r="H46" s="26"/>
-      <c r="I46" s="24"/>
-    </row>
-    <row r="47" spans="1:16" ht="63" customHeight="1">
+      <c r="G46" s="24"/>
+      <c r="H46" s="31"/>
+      <c r="I46" s="26"/>
+      <c r="J46" s="29"/>
+    </row>
+    <row r="47" spans="1:17" ht="63" customHeight="1">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -2511,11 +2601,12 @@
         <v>174</v>
       </c>
       <c r="F47" s="17"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="26"/>
-      <c r="I47" s="24"/>
-    </row>
-    <row r="48" spans="1:16" ht="15.75">
+      <c r="G47" s="24"/>
+      <c r="H47" s="32"/>
+      <c r="I47" s="26"/>
+      <c r="J47" s="29"/>
+    </row>
+    <row r="48" spans="1:17" ht="15.75">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -2532,15 +2623,18 @@
         <v>178</v>
       </c>
       <c r="F48" s="17"/>
-      <c r="G48" s="30" t="s">
+      <c r="G48" s="24" t="s">
         <v>251</v>
       </c>
-      <c r="H48" s="25" t="s">
+      <c r="H48" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="I48" s="25" t="s">
         <v>277</v>
       </c>
-      <c r="I48" s="24"/>
-    </row>
-    <row r="49" spans="1:9" ht="15.75">
+      <c r="J48" s="29"/>
+    </row>
+    <row r="49" spans="1:10" ht="15.75">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -2557,11 +2651,12 @@
         <v>182</v>
       </c>
       <c r="F49" s="17"/>
-      <c r="G49" s="30"/>
-      <c r="H49" s="26"/>
-      <c r="I49" s="24"/>
-    </row>
-    <row r="50" spans="1:9" ht="15.75">
+      <c r="G49" s="24"/>
+      <c r="H49" s="31"/>
+      <c r="I49" s="26"/>
+      <c r="J49" s="29"/>
+    </row>
+    <row r="50" spans="1:10" ht="15.75">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -2578,11 +2673,12 @@
         <v>186</v>
       </c>
       <c r="F50" s="17"/>
-      <c r="G50" s="30"/>
-      <c r="H50" s="26"/>
-      <c r="I50" s="24"/>
-    </row>
-    <row r="51" spans="1:9" ht="15.75">
+      <c r="G50" s="24"/>
+      <c r="H50" s="31"/>
+      <c r="I50" s="26"/>
+      <c r="J50" s="29"/>
+    </row>
+    <row r="51" spans="1:10" ht="15.75">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -2599,11 +2695,12 @@
         <v>190</v>
       </c>
       <c r="F51" s="17"/>
-      <c r="G51" s="30"/>
-      <c r="H51" s="26"/>
-      <c r="I51" s="24"/>
-    </row>
-    <row r="52" spans="1:9" ht="15.75">
+      <c r="G51" s="24"/>
+      <c r="H51" s="31"/>
+      <c r="I51" s="26"/>
+      <c r="J51" s="29"/>
+    </row>
+    <row r="52" spans="1:10" ht="15.75">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -2620,11 +2717,12 @@
         <v>194</v>
       </c>
       <c r="F52" s="17"/>
-      <c r="G52" s="30"/>
-      <c r="H52" s="26"/>
-      <c r="I52" s="24"/>
-    </row>
-    <row r="53" spans="1:9" ht="15.75">
+      <c r="G52" s="24"/>
+      <c r="H52" s="32"/>
+      <c r="I52" s="26"/>
+      <c r="J52" s="29"/>
+    </row>
+    <row r="53" spans="1:10" ht="15.75">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -2641,15 +2739,18 @@
         <v>198</v>
       </c>
       <c r="F53" s="17"/>
-      <c r="G53" s="27" t="s">
+      <c r="G53" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="H53" s="25" t="s">
+      <c r="H53" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="I53" s="25" t="s">
         <v>278</v>
       </c>
-      <c r="I53" s="24"/>
-    </row>
-    <row r="54" spans="1:9" ht="15.75">
+      <c r="J53" s="29"/>
+    </row>
+    <row r="54" spans="1:10" ht="15.75">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -2666,11 +2767,12 @@
         <v>202</v>
       </c>
       <c r="F54" s="17"/>
-      <c r="G54" s="27"/>
-      <c r="H54" s="26"/>
-      <c r="I54" s="24"/>
-    </row>
-    <row r="55" spans="1:9" ht="15.75">
+      <c r="G54" s="24"/>
+      <c r="H54" s="34"/>
+      <c r="I54" s="26"/>
+      <c r="J54" s="29"/>
+    </row>
+    <row r="55" spans="1:10" ht="15.75">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -2687,11 +2789,12 @@
         <v>206</v>
       </c>
       <c r="F55" s="17"/>
-      <c r="G55" s="27"/>
-      <c r="H55" s="26"/>
-      <c r="I55" s="24"/>
-    </row>
-    <row r="56" spans="1:9" ht="15.75">
+      <c r="G55" s="24"/>
+      <c r="H55" s="34"/>
+      <c r="I55" s="26"/>
+      <c r="J55" s="29"/>
+    </row>
+    <row r="56" spans="1:10" ht="15.75">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -2708,11 +2811,12 @@
         <v>210</v>
       </c>
       <c r="F56" s="17"/>
-      <c r="G56" s="27"/>
-      <c r="H56" s="26"/>
-      <c r="I56" s="24"/>
-    </row>
-    <row r="57" spans="1:9" ht="15.75">
+      <c r="G56" s="24"/>
+      <c r="H56" s="34"/>
+      <c r="I56" s="26"/>
+      <c r="J56" s="29"/>
+    </row>
+    <row r="57" spans="1:10" ht="15.75">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -2729,11 +2833,12 @@
         <v>214</v>
       </c>
       <c r="F57" s="17"/>
-      <c r="G57" s="27"/>
-      <c r="H57" s="26"/>
-      <c r="I57" s="24"/>
-    </row>
-    <row r="58" spans="1:9" ht="52.5" customHeight="1">
+      <c r="G57" s="24"/>
+      <c r="H57" s="34"/>
+      <c r="I57" s="26"/>
+      <c r="J57" s="29"/>
+    </row>
+    <row r="58" spans="1:10" ht="52.5" customHeight="1">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -2750,11 +2855,12 @@
         <v>218</v>
       </c>
       <c r="F58" s="17"/>
-      <c r="G58" s="27"/>
-      <c r="H58" s="26"/>
-      <c r="I58" s="24"/>
-    </row>
-    <row r="59" spans="1:9" ht="15.75">
+      <c r="G58" s="24"/>
+      <c r="H58" s="35"/>
+      <c r="I58" s="26"/>
+      <c r="J58" s="29"/>
+    </row>
+    <row r="59" spans="1:10" ht="15.75">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -2771,15 +2877,18 @@
         <v>222</v>
       </c>
       <c r="F59" s="17"/>
-      <c r="G59" s="27" t="s">
+      <c r="G59" s="24" t="s">
         <v>272</v>
       </c>
-      <c r="H59" s="25" t="s">
+      <c r="H59" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="I59" s="25" t="s">
         <v>279</v>
       </c>
-      <c r="I59" s="24"/>
-    </row>
-    <row r="60" spans="1:9" ht="15.75" customHeight="1">
+      <c r="J59" s="29"/>
+    </row>
+    <row r="60" spans="1:10" ht="15.75" customHeight="1">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -2796,11 +2905,12 @@
         <v>226</v>
       </c>
       <c r="F60" s="17"/>
-      <c r="G60" s="27"/>
-      <c r="H60" s="26"/>
-      <c r="I60" s="24"/>
-    </row>
-    <row r="61" spans="1:9" ht="15.75">
+      <c r="G60" s="24"/>
+      <c r="H60" s="34"/>
+      <c r="I60" s="26"/>
+      <c r="J60" s="29"/>
+    </row>
+    <row r="61" spans="1:10" ht="15.75">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -2817,11 +2927,12 @@
         <v>230</v>
       </c>
       <c r="F61" s="17"/>
-      <c r="G61" s="27"/>
-      <c r="H61" s="26"/>
-      <c r="I61" s="24"/>
-    </row>
-    <row r="62" spans="1:9" ht="15.75">
+      <c r="G61" s="24"/>
+      <c r="H61" s="34"/>
+      <c r="I61" s="26"/>
+      <c r="J61" s="29"/>
+    </row>
+    <row r="62" spans="1:10" ht="15.75">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -2838,11 +2949,12 @@
         <v>233</v>
       </c>
       <c r="F62" s="17"/>
-      <c r="G62" s="27"/>
-      <c r="H62" s="26"/>
-      <c r="I62" s="24"/>
-    </row>
-    <row r="63" spans="1:9" ht="15.75">
+      <c r="G62" s="24"/>
+      <c r="H62" s="34"/>
+      <c r="I62" s="26"/>
+      <c r="J62" s="29"/>
+    </row>
+    <row r="63" spans="1:10" ht="15.75">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -2859,11 +2971,12 @@
         <v>237</v>
       </c>
       <c r="F63" s="19"/>
-      <c r="G63" s="27"/>
-      <c r="H63" s="26"/>
-      <c r="I63" s="24"/>
-    </row>
-    <row r="64" spans="1:9" ht="15.75">
+      <c r="G63" s="24"/>
+      <c r="H63" s="34"/>
+      <c r="I63" s="26"/>
+      <c r="J63" s="29"/>
+    </row>
+    <row r="64" spans="1:10" ht="15.75">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -2880,11 +2993,12 @@
         <v>241</v>
       </c>
       <c r="F64" s="19"/>
-      <c r="G64" s="27"/>
-      <c r="H64" s="26"/>
-      <c r="I64" s="24"/>
-    </row>
-    <row r="65" spans="1:9" ht="15.75">
+      <c r="G64" s="24"/>
+      <c r="H64" s="34"/>
+      <c r="I64" s="26"/>
+      <c r="J64" s="29"/>
+    </row>
+    <row r="65" spans="1:10" ht="15.75">
       <c r="A65" s="3">
         <v>64</v>
       </c>
@@ -2897,53 +3011,68 @@
       <c r="D65" s="12"/>
       <c r="E65" s="12"/>
       <c r="F65" s="19"/>
-      <c r="G65" s="27"/>
-      <c r="H65" s="26"/>
-      <c r="I65" s="24"/>
-    </row>
-    <row r="66" spans="1:9" ht="36">
+      <c r="G65" s="24"/>
+      <c r="H65" s="35"/>
+      <c r="I65" s="26"/>
+      <c r="J65" s="29"/>
+    </row>
+    <row r="66" spans="1:10" ht="36">
       <c r="C66" s="14" t="s">
         <v>254</v>
       </c>
       <c r="G66" s="21"/>
       <c r="H66" s="21"/>
-      <c r="I66" s="24"/>
-    </row>
-    <row r="67" spans="1:9" ht="36">
+      <c r="I66" s="21"/>
+      <c r="J66" s="29"/>
+    </row>
+    <row r="67" spans="1:10" ht="36">
       <c r="C67" s="14" t="s">
         <v>255</v>
       </c>
       <c r="G67" s="21"/>
       <c r="H67" s="21"/>
-      <c r="I67" s="24"/>
+      <c r="I67" s="21"/>
+      <c r="J67" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="37">
+    <mergeCell ref="H38:H42"/>
+    <mergeCell ref="H43:H47"/>
+    <mergeCell ref="H48:H52"/>
+    <mergeCell ref="H53:H58"/>
+    <mergeCell ref="H59:H65"/>
+    <mergeCell ref="G7:G11"/>
+    <mergeCell ref="G12:G16"/>
+    <mergeCell ref="J2:J67"/>
+    <mergeCell ref="I33:I37"/>
+    <mergeCell ref="I38:I42"/>
+    <mergeCell ref="I43:I47"/>
+    <mergeCell ref="I48:I52"/>
+    <mergeCell ref="I53:I58"/>
+    <mergeCell ref="I59:I65"/>
+    <mergeCell ref="H2:H6"/>
+    <mergeCell ref="H12:H16"/>
+    <mergeCell ref="H7:H11"/>
+    <mergeCell ref="H17:H21"/>
+    <mergeCell ref="H22:H26"/>
+    <mergeCell ref="H27:H32"/>
+    <mergeCell ref="H33:H37"/>
     <mergeCell ref="G17:G21"/>
     <mergeCell ref="G22:G26"/>
     <mergeCell ref="G53:G58"/>
     <mergeCell ref="G59:G65"/>
-    <mergeCell ref="H2:H6"/>
-    <mergeCell ref="H7:H11"/>
-    <mergeCell ref="H12:H16"/>
-    <mergeCell ref="H17:H21"/>
-    <mergeCell ref="H22:H26"/>
-    <mergeCell ref="H27:H32"/>
+    <mergeCell ref="I2:I6"/>
+    <mergeCell ref="I7:I11"/>
+    <mergeCell ref="I12:I16"/>
+    <mergeCell ref="I17:I21"/>
+    <mergeCell ref="I22:I26"/>
+    <mergeCell ref="I27:I32"/>
     <mergeCell ref="G27:G32"/>
     <mergeCell ref="G33:G37"/>
     <mergeCell ref="G38:G42"/>
     <mergeCell ref="G43:G47"/>
     <mergeCell ref="G48:G52"/>
     <mergeCell ref="G2:G6"/>
-    <mergeCell ref="G7:G11"/>
-    <mergeCell ref="G12:G16"/>
-    <mergeCell ref="I2:I67"/>
-    <mergeCell ref="H33:H37"/>
-    <mergeCell ref="H38:H42"/>
-    <mergeCell ref="H43:H47"/>
-    <mergeCell ref="H48:H52"/>
-    <mergeCell ref="H53:H58"/>
-    <mergeCell ref="H59:H65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>